<commit_message>
Conversion case added as well
</commit_message>
<xml_diff>
--- a/RR_Datasheet.xlsx
+++ b/RR_Datasheet.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SA118193\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E488CE68-A581-493D-B381-87CE329A7B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F944B51D-DDF6-48AF-B3D3-2018FEBFC61A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2F23B69B-FF01-4F36-A027-F39019D388F5}"/>
   </bookViews>
   <sheets>
-    <sheet name="TR" sheetId="1" r:id="rId1"/>
-    <sheet name="RR" sheetId="2" r:id="rId2"/>
+    <sheet name="CV" sheetId="1" r:id="rId1"/>
+    <sheet name="TR" sheetId="3" r:id="rId2"/>
+    <sheet name="RR" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="108">
   <si>
     <t>S.N.O</t>
   </si>
@@ -297,9 +298,6 @@
     <t>Standard Customer Trials</t>
   </si>
   <si>
-    <t>PREMIUM PLUS PLUS</t>
-  </si>
-  <si>
     <t>GPP-0516|01 - BUFFALO CHIEF LINK</t>
   </si>
   <si>
@@ -334,13 +332,43 @@
   </si>
   <si>
     <t>GAMING DEVICE HELIX XT GEN8</t>
+  </si>
+  <si>
+    <t>PREMIUM PLUS</t>
+  </si>
+  <si>
+    <t>Conversions Paid (Serial UnKnown)</t>
+  </si>
+  <si>
+    <t>Game Sales Conversions Only</t>
+  </si>
+  <si>
+    <t>Conversion</t>
+  </si>
+  <si>
+    <t>HELIX XT NO TOPPER BLACK CANDLE EXTENSION</t>
+  </si>
+  <si>
+    <t>BTN PANEL VIRTUAL K1200 HELIX XT</t>
+  </si>
+  <si>
+    <t>Button Panel</t>
+  </si>
+  <si>
+    <t>HELIX XT MAIN VIDEO DISPLAY LCD 43 INCH P-CURVE CLEAR TOUCHSCREEN</t>
+  </si>
+  <si>
+    <t>INSERT BILL NOTE 10-200 ALL HELIX RSA</t>
+  </si>
+  <si>
+    <t>Note: Few Columns are hidden</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -359,7 +387,7 @@
       <sz val="10"/>
       <color rgb="FF212121"/>
       <name val="Segoe UI"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -374,8 +402,15 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -406,6 +441,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -434,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -458,6 +499,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,10 +836,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8B4445C-2A83-4CAD-9CE9-E726F3389DFF}">
-  <dimension ref="A1:AT6"/>
+  <dimension ref="A1:AT7"/>
   <sheetFormatPr defaultColWidth="19.36328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="19.36328125" style="7"/>
+    <col min="1" max="17" width="19.36328125" style="7"/>
+    <col min="18" max="18" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="19" max="22" width="19.36328125" style="7"/>
+    <col min="23" max="23" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="24" max="24" width="19.36328125" style="7"/>
+    <col min="25" max="25" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="19.36328125" style="7"/>
+    <col min="27" max="27" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="19.36328125" style="7"/>
+    <col min="29" max="31" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="32" max="33" width="19.36328125" style="7"/>
+    <col min="34" max="35" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="36" max="36" width="19.36328125" style="7"/>
+    <col min="37" max="38" width="0" style="7" hidden="1" customWidth="1"/>
+    <col min="39" max="16384" width="19.36328125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.35">
@@ -850,9 +908,6 @@
       <c r="Q1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="S1" s="6" t="s">
         <v>16</v>
       </c>
@@ -865,38 +920,27 @@
       <c r="V1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="6" t="s">
-        <v>21</v>
-      </c>
       <c r="X1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="5"/>
+      <c r="Z1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="AA1" s="5"/>
       <c r="AB1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="5" t="s">
-        <v>27</v>
-      </c>
+      <c r="AC1" s="5"/>
       <c r="AD1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="AE1" s="5"/>
       <c r="AF1" s="5" t="s">
         <v>30</v>
       </c>
       <c r="AG1" s="5" t="s">
-        <v>31</v>
+        <v>104</v>
       </c>
       <c r="AH1" s="5" t="s">
         <v>32</v>
@@ -938,7 +982,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:46" ht="48" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:46" ht="59" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -963,92 +1007,70 @@
         <v>49</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>82</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>52</v>
+        <v>101</v>
       </c>
       <c r="N2" s="2">
         <v>2</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>54</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="R2" s="2"/>
+        <v>86</v>
+      </c>
       <c r="S2" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="T2" s="2">
         <v>0.01</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="V2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="X2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y2" s="2"/>
+      <c r="Z2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="Y2" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="AA2" s="2"/>
       <c r="AB2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
+      <c r="AF2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="AE2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AF2" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="AG2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AH2" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="AI2" s="2" t="s">
-        <v>71</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="AH2" s="4"/>
+      <c r="AI2" s="2"/>
       <c r="AJ2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK2" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="AL2" s="2" t="s">
-        <v>74</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="AK2" s="2"/>
+      <c r="AL2" s="2"/>
       <c r="AM2" s="2" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="AN2" s="2" t="s">
         <v>68</v>
@@ -1066,14 +1088,19 @@
         <v>79</v>
       </c>
       <c r="AS2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AT2" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="AT2" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:46" x14ac:dyDescent="0.35">
       <c r="S6" s="8"/>
+    </row>
+    <row r="7" spans="1:46" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>107</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1082,6 +1109,290 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23A908A9-6DF4-4175-8B4A-A57EC672B573}">
+  <dimension ref="A1:AT2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:46" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="T1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="AM1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="AN1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="AQ1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AR1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AT1" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46" s="7" customFormat="1" ht="48" x14ac:dyDescent="0.45">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N2" s="2">
+        <v>2</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="R2" s="2"/>
+      <c r="S2" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="T2" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH2" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AN2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AS2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AT2" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E253A121-1EFD-41EB-AAF1-90E605DA67D7}">
   <dimension ref="A1:AT2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Conversion & Non Gaming ops case added
</commit_message>
<xml_diff>
--- a/RR_Datasheet.xlsx
+++ b/RR_Datasheet.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SA118193\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F944B51D-DDF6-48AF-B3D3-2018FEBFC61A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902E9213-7A06-4217-8BDD-224327FB2DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2F23B69B-FF01-4F36-A027-F39019D388F5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{2F23B69B-FF01-4F36-A027-F39019D388F5}"/>
   </bookViews>
   <sheets>
     <sheet name="CV" sheetId="1" r:id="rId1"/>
     <sheet name="TR" sheetId="3" r:id="rId2"/>
-    <sheet name="RR" sheetId="2" r:id="rId3"/>
+    <sheet name="NG" sheetId="2" r:id="rId3"/>
+    <sheet name="RR" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="117">
   <si>
     <t>S.N.O</t>
   </si>
@@ -362,6 +363,33 @@
   </si>
   <si>
     <t>Note: Few Columns are hidden</t>
+  </si>
+  <si>
+    <t>GREEN VALLEY RANCH RESORT SPA CASINO</t>
+  </si>
+  <si>
+    <t>2300 PASEO VERDE PKWY, HENDERSON, Nevada 89052-2672</t>
+  </si>
+  <si>
+    <t>Non-Gaming Operations</t>
+  </si>
+  <si>
+    <t>Non GOps Fixed Fee</t>
+  </si>
+  <si>
+    <t>TPP000127-LATAM|01 - TOPPER 19.5 INCH LCD HELIX XT LATAM</t>
+  </si>
+  <si>
+    <t>BTN000104|01 - BTN PANEL VIRTUAL K1200 HELIX XT</t>
+  </si>
+  <si>
+    <t>TOPPER 19.5 INCH LCD HELIX XT LATAM</t>
+  </si>
+  <si>
+    <t>BA READY, NO BILL ACCEPTOR PROVIDED HLX VIR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUFFALO CHIEF, VAR 07                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                   </t>
   </si>
 </sst>
 </file>
@@ -475,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -501,6 +529,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -990,8 +1021,8 @@
         <v>45</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="2" t="s">
-        <v>46</v>
+      <c r="D2" s="10" t="s">
+        <v>108</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
@@ -1010,7 +1041,7 @@
         <v>100</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>99</v>
@@ -1397,6 +1428,292 @@
   <dimension ref="A1:AT2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
+    <row r="1" spans="1:46" s="7" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="T1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH1" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="AM1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="AN1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AO1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="AQ1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AR1" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS1" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AT1" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46" s="7" customFormat="1" ht="160.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N2" s="2">
+        <v>2</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="T2" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AB2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AC2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AD2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AF2" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH2" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AL2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AM2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="AN2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AO2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="AR2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="AS2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="AT2" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813209A1-C5EE-4A5F-A03F-162AA894372E}">
+  <dimension ref="A1:AT2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
     <row r="1" spans="1:46" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>

</xml_diff>